<commit_message>
Add circlefilters block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 8
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-asian-paints-safe-painting-service.report.xlsx
+++ b/tools/importer/reports/import-asian-paints-safe-painting-service.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="21">
   <si>
     <t>_reportFile</t>
   </si>
@@ -28,9 +28,6 @@
     <t>timestamp</t>
   </si>
   <si>
-    <t>title</t>
-  </si>
-  <si>
     <t>url</t>
   </si>
   <si>
@@ -49,7 +46,7 @@
     <t>success</t>
   </si>
   <si>
-    <t>2026-10-01T08:39:07.451Z</t>
+    <t>2026-10-02T05:47:20.947Z</t>
   </si>
   <si>
     <t>https://www.asianpaints.com/services/asian-paints-safe-painting-service/interior-paints-and-textures.html</t>
@@ -465,19 +462,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="48" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
     <col min="3" max="3" width="36" customWidth="1"/>
     <col min="5" max="5" width="26" customWidth="1"/>
-    <col min="6" max="6" width="7" customWidth="1"/>
-    <col min="7" max="7" width="50" customWidth="1"/>
-    <col min="8" max="8" width="11" customWidth="1"/>
+    <col min="6" max="6" width="50" customWidth="1"/>
+    <col min="7" max="7" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -499,90 +495,78 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>10</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>11</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>12</v>
-      </c>
-      <c r="F2" t="s">
-        <v>9</v>
       </c>
       <c r="G2" t="s">
         <v>13</v>
       </c>
-      <c r="H2" t="s">
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>14</v>
       </c>
+      <c r="B3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G3" t="s">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>18</v>
       </c>
-      <c r="H3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" t="s">
         <v>19</v>
       </c>
-      <c r="B4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" t="s">
         <v>20</v>
       </c>
-      <c r="D4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" t="s">
-        <v>21</v>
-      </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G4" t="s">
         <v>13</v>
       </c>
-      <c r="H4" t="s">
-        <v>14</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1"/>
+  <autoFilter ref="A1:G1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
refactor: rename circlefilters block to circle-filters
Renames the block folder, files and CSS classes. Published content
still authored as "Circlefilters" is mapped to the renamed block in
scripts.js so existing pages keep rendering. The importer now emits
"Circle Filters" (source selectors still target the AEM .circlefilters).

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-asian-paints-safe-painting-service.report.xlsx
+++ b/tools/importer/reports/import-asian-paints-safe-painting-service.report.xlsx
@@ -11,11 +11,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="22">
   <si>
     <t>_reportFile</t>
   </si>
   <si>
+    <t>circle-filters</t>
+  </si>
+  <si>
     <t>circlefilters</t>
   </si>
   <si>
@@ -40,19 +43,19 @@
     <t>found</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>asian-paints-safe-painting-service</t>
   </si>
   <si>
     <t>success</t>
   </si>
   <si>
-    <t>2026-10-02T06:12:25.147Z</t>
+    <t>2026-10-02T06:24:53.043Z</t>
   </si>
   <si>
     <t>https://www.asianpaints.com/services/asian-paints-safe-painting-service/interior-paints-and-textures.html</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>products.report.json</t>
@@ -462,18 +465,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="48" customWidth="1"/>
-    <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="36" customWidth="1"/>
-    <col min="5" max="5" width="26" customWidth="1"/>
-    <col min="6" max="6" width="50" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="4" max="4" width="36" customWidth="1"/>
+    <col min="6" max="6" width="26" customWidth="1"/>
+    <col min="7" max="7" width="50" customWidth="1"/>
+    <col min="8" max="8" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -495,78 +499,90 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" t="s">
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" t="s">
         <v>12</v>
-      </c>
-      <c r="G2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" t="s">
-        <v>16</v>
       </c>
       <c r="F3" t="s">
         <v>17</v>
       </c>
       <c r="G3" t="s">
-        <v>8</v>
+        <v>18</v>
+      </c>
+      <c r="H3" t="s">
+        <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="D4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" t="s">
+        <v>21</v>
+      </c>
+      <c r="G4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H4" t="s">
         <v>10</v>
-      </c>
-      <c r="E4" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G4" t="s">
-        <v>13</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G1"/>
+  <autoFilter ref="A1:H1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(choose-plan): start v2 slider dots on the first plan; import plans
The v2 dots could mark the last plan as current when the block script ran
before its CSS (row not scrollable yet). A non-scrollable row now counts as
the first plan, and a ResizeObserver re-checks when the layout changes.

The safe-painting-service importer now adds the choose-plan-v2 plans in
their own section after circle-filters (new parsers/choose-plan.js).

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-asian-paints-safe-painting-service.report.xlsx
+++ b/tools/importer/reports/import-asian-paints-safe-painting-service.report.xlsx
@@ -11,17 +11,23 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="28">
   <si>
     <t>_reportFile</t>
   </si>
   <si>
+    <t>choose-plan</t>
+  </si>
+  <si>
     <t>circle-filters</t>
   </si>
   <si>
     <t>circlefilters</t>
   </si>
   <si>
+    <t>explore-store</t>
+  </si>
+  <si>
     <t>path</t>
   </si>
   <si>
@@ -52,7 +58,7 @@
     <t>success</t>
   </si>
   <si>
-    <t>2026-10-02T06:24:53.043Z</t>
+    <t>2026-10-03T08:35:16.752Z</t>
   </si>
   <si>
     <t>https://www.asianpaints.com/services/asian-paints-safe-painting-service/interior-paints-and-textures.html</t>
@@ -77,6 +83,18 @@
   </si>
   <si>
     <t>2026-10-01T07:54:40.112Z</t>
+  </si>
+  <si>
+    <t>store-locator.report.json</t>
+  </si>
+  <si>
+    <t>store-locator</t>
+  </si>
+  <si>
+    <t>2026-10-03T06:49:53.308Z</t>
+  </si>
+  <si>
+    <t>https://www.asianpaints.com/store-locator.html</t>
   </si>
 </sst>
 </file>
@@ -465,19 +483,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="48" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="36" customWidth="1"/>
-    <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="50" customWidth="1"/>
-    <col min="8" max="8" width="11" customWidth="1"/>
+    <col min="2" max="2" width="13" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="15" customWidth="1"/>
+    <col min="6" max="6" width="36" customWidth="1"/>
+    <col min="8" max="8" width="26" customWidth="1"/>
+    <col min="9" max="9" width="50" customWidth="1"/>
+    <col min="10" max="10" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -502,19 +521,25 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E2" t="s">
         <v>12</v>
@@ -526,63 +551,113 @@
         <v>14</v>
       </c>
       <c r="H2" t="s">
-        <v>10</v>
+        <v>15</v>
+      </c>
+      <c r="I2" t="s">
+        <v>16</v>
+      </c>
+      <c r="J2" t="s">
+        <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D3" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E3" t="s">
         <v>12</v>
       </c>
       <c r="F3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G3" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="H3" t="s">
-        <v>9</v>
+        <v>19</v>
+      </c>
+      <c r="I3" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C4" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D4" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="E4" t="s">
         <v>12</v>
       </c>
       <c r="F4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G4" t="s">
         <v>14</v>
       </c>
       <c r="H4" t="s">
-        <v>10</v>
+        <v>23</v>
+      </c>
+      <c r="I4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G5" t="s">
+        <v>14</v>
+      </c>
+      <c r="H5" t="s">
+        <v>26</v>
+      </c>
+      <c r="I5" t="s">
+        <v>27</v>
+      </c>
+      <c r="J5" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1"/>
+  <autoFilter ref="A1:J1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>